<commit_message>
fix: change sample import student to class
</commit_message>
<xml_diff>
--- a/public/files/import_student_to_class.xlsx
+++ b/public/files/import_student_to_class.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="30240" windowHeight="14440"/>
+    <workbookView windowWidth="27945" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Student_Import_-_Template" sheetId="1" r:id="rId1"/>
@@ -44,13 +44,13 @@
     <t>HS0001</t>
   </si>
   <si>
-    <t>thanh hoa2</t>
+    <t>Nguyen Van A</t>
   </si>
   <si>
-    <t>HS0002</t>
+    <t>0123456789</t>
   </si>
   <si>
-    <t>nam dinh2</t>
+    <t>0987654321</t>
   </si>
 </sst>
 </file>
@@ -58,10 +58,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -524,16 +524,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -668,6 +668,9 @@
   </cellStyleXfs>
   <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -683,7 +686,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1203,11 +1206,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="16.8" outlineLevelRow="2" outlineLevelCol="3"/>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.1047619047619" customWidth="1"/>
+    <col min="2" max="2" width="14.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="11.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="13.552380952381" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -1224,19 +1229,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="D2" s="1" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>